<commit_message>
snow user schema integrated
</commit_message>
<xml_diff>
--- a/shift_roster.xlsx
+++ b/shift_roster.xlsx
@@ -2,22 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
   <sheets>
     <sheet name="Shift_Definitions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Associate_Skills" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="MFT" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ESB" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Azure" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Database" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ETL" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="IT_support" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Admin" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Infrastructure" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Developers" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="HR" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="L1_Support" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -57,9 +53,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -206,6 +202,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -240,6 +237,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -274,20 +272,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -409,7 +403,46 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
@@ -421,7 +454,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.57142857142857" customWidth="1" min="1" max="24"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -484,7 +520,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
@@ -494,8 +531,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.57142857142857" customWidth="1" min="1" max="25"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -510,6 +550,11 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Skills</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Skill Level</t>
         </is>
       </c>
@@ -517,15 +562,20 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Alice Smith</t>
+          <t>Naomi Greenly</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>MFT</t>
+          <t>IT support</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
+        <is>
+          <t>Technical Troubleshooting, Operating Systems, Ticketing Systems, Customer Service, Networking Basics</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>L1</t>
         </is>
@@ -534,15 +584,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bob Jones</t>
+          <t>Melinda Carleton</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MFT</t>
+          <t>IT support</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
+        <is>
+          <t>Technical Troubleshooting, Operating Systems, Ticketing Systems, Customer Service, Networking Basics</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>L2</t>
         </is>
@@ -551,15 +606,20 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Charlie Brown</t>
+          <t>Geri Forness</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MFT</t>
+          <t>IT support</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
+        <is>
+          <t>Technical Troubleshooting, Operating Systems, Ticketing Systems, Customer Service, Networking Basics</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
         <is>
           <t>L3</t>
         </is>
@@ -568,15 +628,20 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>David Miller</t>
+          <t>Justina Dragaj</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ESB</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
+        <is>
+          <t>User Management, Backup and Disaster Recovery, Scripting &amp; Automation, Security Compliance, Vendor Management</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
         <is>
           <t>L1</t>
         </is>
@@ -585,15 +650,20 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Emma Wilson</t>
+          <t>Jacinto Gawron</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ESB</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
+        <is>
+          <t>User Management, Backup and Disaster Recovery, Scripting &amp; Automation, Security Compliance, Vendor Management</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>L2</t>
         </is>
@@ -602,15 +672,20 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Frank Thomas</t>
+          <t>Jewel Agresta</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ESB</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
+        <is>
+          <t>User Management, Backup and Disaster Recovery, Scripting &amp; Automation, Security Compliance, Vendor Management</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>L3</t>
         </is>
@@ -619,15 +694,20 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Grace Taylor</t>
+          <t>Tom Diggins-Barnes</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Azure</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
+        <is>
+          <t>Cloud Computing, Networking &amp; Security, Containerization &amp; Orchestration, Infrastructure as Code, Monitoring &amp; Logging</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
         <is>
           <t>L1</t>
         </is>
@@ -636,15 +716,20 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Henry Anderson</t>
+          <t>Jess Assad</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Azure</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
+        <is>
+          <t>Cloud Computing, Networking &amp; Security, Containerization &amp; Orchestration, Infrastructure as Code, Monitoring &amp; Logging</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
         <is>
           <t>L2</t>
         </is>
@@ -653,15 +738,20 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ivy Martin</t>
+          <t>Krystle Stika</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Azure</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
+        <is>
+          <t>Cloud Computing, Networking &amp; Security, Containerization &amp; Orchestration, Infrastructure as Code, Monitoring &amp; Logging</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
         <is>
           <t>L3</t>
         </is>
@@ -670,15 +760,20 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Jack White</t>
+          <t>Sean Bonnet</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Database</t>
+          <t>Developers</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
+        <is>
+          <t>Programming Languages, API Design &amp; Integration, Version Control, Database Management, Testing &amp; Debugging</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
         <is>
           <t>L1</t>
         </is>
@@ -687,15 +782,20 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Kelly Harris</t>
+          <t>Cherie Fuhri</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Database</t>
+          <t>Developers</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
+        <is>
+          <t>Programming Languages, API Design &amp; Integration, Version Control, Database Management, Testing &amp; Debugging</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
         <is>
           <t>L2</t>
         </is>
@@ -704,15 +804,20 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Liam Clark</t>
+          <t>Lucius Bagnoli</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Database</t>
+          <t>Developers</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
+        <is>
+          <t>Programming Languages, API Design &amp; Integration, Version Control, Database Management, Testing &amp; Debugging</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
         <is>
           <t>L3</t>
         </is>
@@ -721,15 +826,20 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mia Lewis</t>
+          <t>Christian Marnell</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ETL</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
+        <is>
+          <t>Talent Acquisition, Employee Relations, Compliance &amp; Employment Law, HRIS Management, Communication &amp; Empathy</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
         <is>
           <t>L1</t>
         </is>
@@ -738,15 +848,20 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Noah Walker</t>
+          <t>Nelly Jakuboski</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ETL</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
+        <is>
+          <t>Talent Acquisition, Employee Relations, Compliance &amp; Employment Law, HRIS Management, Communication &amp; Empathy</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
         <is>
           <t>L2</t>
         </is>
@@ -755,15 +870,20 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Olivia Hall</t>
+          <t>survey user</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ETL</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
+        <is>
+          <t>Talent Acquisition, Employee Relations, Compliance &amp; Employment Law, HRIS Management, Communication &amp; Empathy</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
         <is>
           <t>L3</t>
         </is>
@@ -772,7 +892,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Sophia Allen</t>
+          <t>Jimmie Barninger</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -781,6 +901,11 @@
         </is>
       </c>
       <c r="C17" t="inlineStr">
+        <is>
+          <t>Incident Triage, Basic Diagnostics, Active Listening, Documentation, Knowledge Base Navigation</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
         <is>
           <t>L1</t>
         </is>
@@ -789,7 +914,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>William Young</t>
+          <t>Billie Cowley</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -798,6 +923,11 @@
         </is>
       </c>
       <c r="C18" t="inlineStr">
+        <is>
+          <t>Incident Triage, Basic Diagnostics, Active Listening, Documentation, Knowledge Base Navigation</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
         <is>
           <t>L2</t>
         </is>
@@ -806,7 +936,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Zoe King</t>
+          <t>Dwain Cuttitta</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -816,12 +946,18 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>Incident Triage, Basic Diagnostics, Active Listening, Documentation, Knowledge Base Navigation</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
           <t>L3</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
@@ -832,7 +968,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AF4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.57142857142857" customWidth="1" min="1" max="32"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -840,166 +979,104 @@
           <t>Associate Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
+      <c r="B1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E1" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1" t="n">
+        <v>6</v>
+      </c>
+      <c r="H1" t="n">
+        <v>7</v>
+      </c>
+      <c r="I1" t="n">
+        <v>8</v>
+      </c>
+      <c r="J1" t="n">
+        <v>9</v>
+      </c>
+      <c r="K1" t="n">
+        <v>10</v>
+      </c>
+      <c r="L1" t="n">
+        <v>11</v>
+      </c>
+      <c r="M1" t="n">
+        <v>12</v>
+      </c>
+      <c r="N1" t="n">
+        <v>13</v>
+      </c>
+      <c r="O1" t="n">
+        <v>14</v>
+      </c>
+      <c r="P1" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="n">
+        <v>16</v>
+      </c>
+      <c r="R1" t="n">
+        <v>17</v>
+      </c>
+      <c r="S1" t="n">
+        <v>18</v>
+      </c>
+      <c r="T1" t="n">
+        <v>19</v>
+      </c>
+      <c r="U1" t="n">
+        <v>20</v>
+      </c>
+      <c r="V1" t="n">
+        <v>21</v>
+      </c>
+      <c r="W1" t="n">
+        <v>22</v>
+      </c>
+      <c r="X1" t="n">
+        <v>23</v>
+      </c>
+      <c r="Y1" t="n">
+        <v>24</v>
+      </c>
+      <c r="Z1" t="n">
+        <v>25</v>
+      </c>
+      <c r="AA1" t="n">
+        <v>26</v>
+      </c>
+      <c r="AB1" t="n">
+        <v>27</v>
+      </c>
+      <c r="AC1" t="n">
+        <v>28</v>
+      </c>
+      <c r="AD1" t="n">
+        <v>29</v>
+      </c>
+      <c r="AE1" t="n">
+        <v>30</v>
+      </c>
+      <c r="AF1" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Alice Smith</t>
+          <t>Naomi Greenly</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1161,7 +1238,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bob Jones</t>
+          <t>Melinda Carleton</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1323,7 +1400,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Charlie Brown</t>
+          <t>Geri Forness</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1483,7 +1560,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
@@ -1494,7 +1572,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AF4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.57142857142857" customWidth="1" min="1" max="32"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1502,166 +1583,104 @@
           <t>Associate Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
+      <c r="B1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E1" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1" t="n">
+        <v>6</v>
+      </c>
+      <c r="H1" t="n">
+        <v>7</v>
+      </c>
+      <c r="I1" t="n">
+        <v>8</v>
+      </c>
+      <c r="J1" t="n">
+        <v>9</v>
+      </c>
+      <c r="K1" t="n">
+        <v>10</v>
+      </c>
+      <c r="L1" t="n">
+        <v>11</v>
+      </c>
+      <c r="M1" t="n">
+        <v>12</v>
+      </c>
+      <c r="N1" t="n">
+        <v>13</v>
+      </c>
+      <c r="O1" t="n">
+        <v>14</v>
+      </c>
+      <c r="P1" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="n">
+        <v>16</v>
+      </c>
+      <c r="R1" t="n">
+        <v>17</v>
+      </c>
+      <c r="S1" t="n">
+        <v>18</v>
+      </c>
+      <c r="T1" t="n">
+        <v>19</v>
+      </c>
+      <c r="U1" t="n">
+        <v>20</v>
+      </c>
+      <c r="V1" t="n">
+        <v>21</v>
+      </c>
+      <c r="W1" t="n">
+        <v>22</v>
+      </c>
+      <c r="X1" t="n">
+        <v>23</v>
+      </c>
+      <c r="Y1" t="n">
+        <v>24</v>
+      </c>
+      <c r="Z1" t="n">
+        <v>25</v>
+      </c>
+      <c r="AA1" t="n">
+        <v>26</v>
+      </c>
+      <c r="AB1" t="n">
+        <v>27</v>
+      </c>
+      <c r="AC1" t="n">
+        <v>28</v>
+      </c>
+      <c r="AD1" t="n">
+        <v>29</v>
+      </c>
+      <c r="AE1" t="n">
+        <v>30</v>
+      </c>
+      <c r="AF1" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>David Miller</t>
+          <t>Justina Dragaj</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1823,7 +1842,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Emma Wilson</t>
+          <t>Jacinto Gawron</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1985,7 +2004,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Frank Thomas</t>
+          <t>Jewel Agresta</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2145,7 +2164,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
@@ -2156,7 +2176,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AF4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.57142857142857" customWidth="1" min="1" max="32"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2164,166 +2187,104 @@
           <t>Associate Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
+      <c r="B1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E1" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1" t="n">
+        <v>6</v>
+      </c>
+      <c r="H1" t="n">
+        <v>7</v>
+      </c>
+      <c r="I1" t="n">
+        <v>8</v>
+      </c>
+      <c r="J1" t="n">
+        <v>9</v>
+      </c>
+      <c r="K1" t="n">
+        <v>10</v>
+      </c>
+      <c r="L1" t="n">
+        <v>11</v>
+      </c>
+      <c r="M1" t="n">
+        <v>12</v>
+      </c>
+      <c r="N1" t="n">
+        <v>13</v>
+      </c>
+      <c r="O1" t="n">
+        <v>14</v>
+      </c>
+      <c r="P1" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="n">
+        <v>16</v>
+      </c>
+      <c r="R1" t="n">
+        <v>17</v>
+      </c>
+      <c r="S1" t="n">
+        <v>18</v>
+      </c>
+      <c r="T1" t="n">
+        <v>19</v>
+      </c>
+      <c r="U1" t="n">
+        <v>20</v>
+      </c>
+      <c r="V1" t="n">
+        <v>21</v>
+      </c>
+      <c r="W1" t="n">
+        <v>22</v>
+      </c>
+      <c r="X1" t="n">
+        <v>23</v>
+      </c>
+      <c r="Y1" t="n">
+        <v>24</v>
+      </c>
+      <c r="Z1" t="n">
+        <v>25</v>
+      </c>
+      <c r="AA1" t="n">
+        <v>26</v>
+      </c>
+      <c r="AB1" t="n">
+        <v>27</v>
+      </c>
+      <c r="AC1" t="n">
+        <v>28</v>
+      </c>
+      <c r="AD1" t="n">
+        <v>29</v>
+      </c>
+      <c r="AE1" t="n">
+        <v>30</v>
+      </c>
+      <c r="AF1" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Grace Taylor</t>
+          <t>Tom Diggins-Barnes</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2485,7 +2446,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Henry Anderson</t>
+          <t>Jess Assad</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2647,7 +2608,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ivy Martin</t>
+          <t>Krystle Stika</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2807,7 +2768,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
@@ -2818,7 +2780,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AF4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.57142857142857" customWidth="1" min="1" max="32"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2826,166 +2791,104 @@
           <t>Associate Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
+      <c r="B1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E1" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1" t="n">
+        <v>6</v>
+      </c>
+      <c r="H1" t="n">
+        <v>7</v>
+      </c>
+      <c r="I1" t="n">
+        <v>8</v>
+      </c>
+      <c r="J1" t="n">
+        <v>9</v>
+      </c>
+      <c r="K1" t="n">
+        <v>10</v>
+      </c>
+      <c r="L1" t="n">
+        <v>11</v>
+      </c>
+      <c r="M1" t="n">
+        <v>12</v>
+      </c>
+      <c r="N1" t="n">
+        <v>13</v>
+      </c>
+      <c r="O1" t="n">
+        <v>14</v>
+      </c>
+      <c r="P1" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="n">
+        <v>16</v>
+      </c>
+      <c r="R1" t="n">
+        <v>17</v>
+      </c>
+      <c r="S1" t="n">
+        <v>18</v>
+      </c>
+      <c r="T1" t="n">
+        <v>19</v>
+      </c>
+      <c r="U1" t="n">
+        <v>20</v>
+      </c>
+      <c r="V1" t="n">
+        <v>21</v>
+      </c>
+      <c r="W1" t="n">
+        <v>22</v>
+      </c>
+      <c r="X1" t="n">
+        <v>23</v>
+      </c>
+      <c r="Y1" t="n">
+        <v>24</v>
+      </c>
+      <c r="Z1" t="n">
+        <v>25</v>
+      </c>
+      <c r="AA1" t="n">
+        <v>26</v>
+      </c>
+      <c r="AB1" t="n">
+        <v>27</v>
+      </c>
+      <c r="AC1" t="n">
+        <v>28</v>
+      </c>
+      <c r="AD1" t="n">
+        <v>29</v>
+      </c>
+      <c r="AE1" t="n">
+        <v>30</v>
+      </c>
+      <c r="AF1" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Jack White</t>
+          <t>Sean Bonnet</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3147,7 +3050,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Kelly Harris</t>
+          <t>Cherie Fuhri</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3309,7 +3212,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Liam Clark</t>
+          <t>Lucius Bagnoli</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3469,7 +3372,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
@@ -3480,7 +3384,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AF4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.57142857142857" customWidth="1" min="1" max="32"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -3488,166 +3395,104 @@
           <t>Associate Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
+      <c r="B1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E1" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1" t="n">
+        <v>6</v>
+      </c>
+      <c r="H1" t="n">
+        <v>7</v>
+      </c>
+      <c r="I1" t="n">
+        <v>8</v>
+      </c>
+      <c r="J1" t="n">
+        <v>9</v>
+      </c>
+      <c r="K1" t="n">
+        <v>10</v>
+      </c>
+      <c r="L1" t="n">
+        <v>11</v>
+      </c>
+      <c r="M1" t="n">
+        <v>12</v>
+      </c>
+      <c r="N1" t="n">
+        <v>13</v>
+      </c>
+      <c r="O1" t="n">
+        <v>14</v>
+      </c>
+      <c r="P1" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="n">
+        <v>16</v>
+      </c>
+      <c r="R1" t="n">
+        <v>17</v>
+      </c>
+      <c r="S1" t="n">
+        <v>18</v>
+      </c>
+      <c r="T1" t="n">
+        <v>19</v>
+      </c>
+      <c r="U1" t="n">
+        <v>20</v>
+      </c>
+      <c r="V1" t="n">
+        <v>21</v>
+      </c>
+      <c r="W1" t="n">
+        <v>22</v>
+      </c>
+      <c r="X1" t="n">
+        <v>23</v>
+      </c>
+      <c r="Y1" t="n">
+        <v>24</v>
+      </c>
+      <c r="Z1" t="n">
+        <v>25</v>
+      </c>
+      <c r="AA1" t="n">
+        <v>26</v>
+      </c>
+      <c r="AB1" t="n">
+        <v>27</v>
+      </c>
+      <c r="AC1" t="n">
+        <v>28</v>
+      </c>
+      <c r="AD1" t="n">
+        <v>29</v>
+      </c>
+      <c r="AE1" t="n">
+        <v>30</v>
+      </c>
+      <c r="AF1" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Mia Lewis</t>
+          <t>Christian Marnell</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3809,7 +3654,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Noah Walker</t>
+          <t>Nelly Jakuboski</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3971,7 +3816,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Olivia Hall</t>
+          <t>survey user</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4131,7 +3976,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
@@ -4142,7 +3988,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AF4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.57142857142857" customWidth="1" min="1" max="32"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -4150,166 +3999,104 @@
           <t>Associate Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
+      <c r="B1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E1" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1" t="n">
+        <v>6</v>
+      </c>
+      <c r="H1" t="n">
+        <v>7</v>
+      </c>
+      <c r="I1" t="n">
+        <v>8</v>
+      </c>
+      <c r="J1" t="n">
+        <v>9</v>
+      </c>
+      <c r="K1" t="n">
+        <v>10</v>
+      </c>
+      <c r="L1" t="n">
+        <v>11</v>
+      </c>
+      <c r="M1" t="n">
+        <v>12</v>
+      </c>
+      <c r="N1" t="n">
+        <v>13</v>
+      </c>
+      <c r="O1" t="n">
+        <v>14</v>
+      </c>
+      <c r="P1" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="n">
+        <v>16</v>
+      </c>
+      <c r="R1" t="n">
+        <v>17</v>
+      </c>
+      <c r="S1" t="n">
+        <v>18</v>
+      </c>
+      <c r="T1" t="n">
+        <v>19</v>
+      </c>
+      <c r="U1" t="n">
+        <v>20</v>
+      </c>
+      <c r="V1" t="n">
+        <v>21</v>
+      </c>
+      <c r="W1" t="n">
+        <v>22</v>
+      </c>
+      <c r="X1" t="n">
+        <v>23</v>
+      </c>
+      <c r="Y1" t="n">
+        <v>24</v>
+      </c>
+      <c r="Z1" t="n">
+        <v>25</v>
+      </c>
+      <c r="AA1" t="n">
+        <v>26</v>
+      </c>
+      <c r="AB1" t="n">
+        <v>27</v>
+      </c>
+      <c r="AC1" t="n">
+        <v>28</v>
+      </c>
+      <c r="AD1" t="n">
+        <v>29</v>
+      </c>
+      <c r="AE1" t="n">
+        <v>30</v>
+      </c>
+      <c r="AF1" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sophia Allen</t>
+          <t>Jimmie Barninger</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4471,7 +4258,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>William Young</t>
+          <t>Billie Cowley</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4633,7 +4420,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Zoe King</t>
+          <t>Dwain Cuttitta</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4793,6 +4580,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>